<commit_message>
Added category, service update, working hours and manpower
</commit_message>
<xml_diff>
--- a/data/complaints.xlsx
+++ b/data/complaints.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,25 +453,50 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Breakdown Type</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Reported By</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Assigned To</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Assigned Person</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Working Hours</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Manpower</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Service Remark</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Image Path</t>
         </is>
@@ -480,20 +505,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CI-20260731-001</t>
+          <t>CI-20260803-001</t>
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Oxygen Plant</t>
+          <t>SMS-1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AI-101</t>
+          <t>PT-01</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -508,131 +533,46 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>Instrumentation</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Epsita</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>Jeet</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>Instrumentation Team</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jitendra Rade</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>complaints_images/CI-20260731-001_1.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CI-20260801-002</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="n">
-        <v>46235</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Pellet Plant</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>ABCD</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>TT is not working</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Process</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Jeet</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Instrumentation Team</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CI-20260801-003</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="n">
-        <v>46235</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Pellet Plant</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>ABCD</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>TT is not working</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Process</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Jeet</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Instrumentation Team</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added complaint registration improvements and Gmail SMTP email notification
</commit_message>
<xml_diff>
--- a/data/complaints.xlsx
+++ b/data/complaints.xlsx
@@ -16,9 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,9 +51,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:S12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,30 +476,45 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>HOD</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Target Date</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>HOD Remark</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>Assigned Person</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Working Hours</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Manpower</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Service Remark</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Image Path</t>
         </is>
@@ -505,74 +523,849 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CI-20260803-001</t>
+          <t>CI-20260806-001</t>
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46237</v>
+        <v>46240</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SMS-1</t>
+          <t>Power Plant (3x130MW)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>AI-101</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>not workin</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Epsita</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Avhinash Ujjwal</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CI-20260806-002</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Power Plant (3x130MW)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>AI-101</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>not workin</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Epsita</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Avhinash Ujjwal</t>
+        </is>
+      </c>
+      <c r="L3" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CI-20260806-003</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Power Plant (3x130MW)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>AI-101</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>not working</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Epsita</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Avhinash Ujjwal</t>
+        </is>
+      </c>
+      <c r="L4" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CI-20260806-004</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Power Plant (3x130MW)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AI-101</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>not working</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Epsita</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Avhinash Ujjwal</t>
+        </is>
+      </c>
+      <c r="L5" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CI-20260806-005</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Power Plant (3x130MW)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>AI-101</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>not working</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Epsita</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Avhinash Ujjwal</t>
+        </is>
+      </c>
+      <c r="L6" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CI-20260806-006</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Power Plant (3x130MW)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AI-101</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>not working</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Epsita</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Avhinash Ujjwal</t>
+        </is>
+      </c>
+      <c r="L7" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CI-20260806-007</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Power Plant (3x130MW)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>AI-101</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>not working</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Epsita</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Avhinash Ujjwal</t>
+        </is>
+      </c>
+      <c r="L8" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CI-20260806-008</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Power Plant (3x130MW)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>AI-101</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>not working</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Epsita</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Avhinash Ujjwal</t>
+        </is>
+      </c>
+      <c r="L9" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CI-20260806-009</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Power Plant (3x130MW)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>AI-101</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>not working</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Epsita</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Avhinash Ujjwal</t>
+        </is>
+      </c>
+      <c r="L10" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CI-20260806-010</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Power Plant (3x130MW)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>PT-01</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Not ok</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Not working</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Calibration</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Instrumentation</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>Jeet</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Instrumentation Team</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jitendra Rade</t>
-        </is>
-      </c>
-      <c r="L2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Avhinash Ujjwal</t>
+        </is>
+      </c>
+      <c r="L11" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CI-20260806-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Power Plant (3x130MW)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PT-01</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Not working</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Jeet</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Avhinash Ujjwal</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Updated professional header for complaint list
</commit_message>
<xml_diff>
--- a/data/complaints.xlsx
+++ b/data/complaints.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -512,6 +516,83 @@
           <t>Image Path</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CI-20260808-001</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Power Plant (3x130MW)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>pt-101</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Not working</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Epsita</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Avhinash Ujjwal</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>